<commit_message>
Condense both courses into fewer, concept-based, illustrated lectures
Radiative Transfer now has 6 lectures (RT1-RT6) plus exam and formula
sheet; Stellar Atmospheres has 5 (SA1-SA5) plus exam and formula sheet.
Each lecture opens with a concept map, explains the big ideas in plain
words before the mathematics, and keeps the best verified worked
examples, four misconceptions, a summary and four exam Q&As.

New illustrations: eleven concept maps, flux vs intensity, the four
light-matter interactions, the contribution function, TE/LTE/NLTE
pictured, where a line forms, and Novotny's three-step hand-built solar
model atmosphere (new worked example and sa_physics helpers). Cross-
references, app labels, spreadsheet sheets, README and title pages are
renumbered; figure captions get their own CSS class in the PDF build.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Lb5cDd29sk38kzcehHJCfg
</commit_message>
<xml_diff>
--- a/Radiative_Transfer_Lab.xlsx
+++ b/Radiative_Transfer_Lab.xlsx
@@ -2,23 +2,23 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <fileVersion appName="Calc"/>
-  <workbookPr backupFile="false" showObjects="all" date1904="false"/>
+  <workbookPr backupFile="false" showObjects="all" dateCompatibility="false"/>
   <workbookProtection/>
   <bookViews>
-    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="0"/>
+    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="600" firstSheet="0" activeTab="0"/>
   </bookViews>
   <sheets>
     <sheet name="Start here" sheetId="1" state="visible" r:id="rId3"/>
     <sheet name="RT1 Optical depth" sheetId="2" state="visible" r:id="rId4"/>
-    <sheet name="RT2 Intensity" sheetId="3" state="visible" r:id="rId5"/>
-    <sheet name="RT3 Planck" sheetId="4" state="visible" r:id="rId6"/>
-    <sheet name="RT4 Random walk" sheetId="5" state="visible" r:id="rId7"/>
-    <sheet name="RT5 Slab &amp; MIT star" sheetId="6" state="visible" r:id="rId8"/>
+    <sheet name="RT1 Intensity" sheetId="3" state="visible" r:id="rId5"/>
+    <sheet name="RT2 Planck" sheetId="4" state="visible" r:id="rId6"/>
+    <sheet name="RT2 Random walk" sheetId="5" state="visible" r:id="rId7"/>
+    <sheet name="RT3 Slab &amp; MIT star" sheetId="6" state="visible" r:id="rId8"/>
     <sheet name="SA1 Saha-Boltzmann" sheetId="7" state="visible" r:id="rId9"/>
-    <sheet name="RT7 Eddington-Barbier" sheetId="8" state="visible" r:id="rId10"/>
-    <sheet name="RT8 Scattering" sheetId="9" state="visible" r:id="rId11"/>
-    <sheet name="SA5 Gray atmosphere" sheetId="10" state="visible" r:id="rId12"/>
-    <sheet name="SA6 Lines" sheetId="11" state="visible" r:id="rId13"/>
+    <sheet name="RT4 Eddington-Barbier" sheetId="8" state="visible" r:id="rId10"/>
+    <sheet name="RT4 Scattering" sheetId="9" state="visible" r:id="rId11"/>
+    <sheet name="SA4 Gray atmosphere" sheetId="10" state="visible" r:id="rId12"/>
+    <sheet name="SA4 Lines" sheetId="11" state="visible" r:id="rId13"/>
     <sheet name="Constants" sheetId="12" state="visible" r:id="rId14"/>
     <sheet name="Data" sheetId="13" state="visible" r:id="rId15"/>
   </sheets>
@@ -49,7 +49,7 @@
 </file>
 
 <file path=xl/comments10.xml><?xml version="1.0" encoding="utf-8"?>
-<comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
+<comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:v2="http://schemas.openxmlformats.org/spreadsheetml/2006/main/v2" mc:Ignorable="v2">
   <authors>
     <author>Unknown Author</author>
   </authors>
@@ -65,6 +65,27 @@
           <t xml:space="preserve">Sun 5772 K. The gray solution is self-similar in T/T_eff.</t>
         </r>
       </text>
+      <mc:AlternateContent>
+        <mc:Choice Requires="v2">
+          <commentPr autoFill="true" autoScale="false" colHidden="false" locked="false" rowHidden="false" textHAlign="justify" textVAlign="top">
+            <anchor moveWithCells="false" sizeWithCells="false">
+              <xdr:from>
+                <xdr:col>0</xdr:col>
+                <xdr:colOff>79</xdr:colOff>
+                <xdr:row>0</xdr:row>
+                <xdr:rowOff>5</xdr:rowOff>
+              </xdr:from>
+              <xdr:to>
+                <xdr:col>1</xdr:col>
+                <xdr:colOff>-58</xdr:colOff>
+                <xdr:row>4</xdr:row>
+                <xdr:rowOff>1</xdr:rowOff>
+              </xdr:to>
+            </anchor>
+          </commentPr>
+        </mc:Choice>
+        <mc:Fallback/>
+      </mc:AlternateContent>
     </comment>
     <comment ref="B7" authorId="0">
       <text>
@@ -77,6 +98,27 @@
           <t xml:space="preserve">Compare 300 nm (strong darkening) with 1500 nm.</t>
         </r>
       </text>
+      <mc:AlternateContent>
+        <mc:Choice Requires="v2">
+          <commentPr autoFill="true" autoScale="false" colHidden="false" locked="false" rowHidden="false" textHAlign="justify" textVAlign="top">
+            <anchor moveWithCells="false" sizeWithCells="false">
+              <xdr:from>
+                <xdr:col>0</xdr:col>
+                <xdr:colOff>79</xdr:colOff>
+                <xdr:row>0</xdr:row>
+                <xdr:rowOff>5</xdr:rowOff>
+              </xdr:from>
+              <xdr:to>
+                <xdr:col>1</xdr:col>
+                <xdr:colOff>-58</xdr:colOff>
+                <xdr:row>4</xdr:row>
+                <xdr:rowOff>1</xdr:rowOff>
+              </xdr:to>
+            </anchor>
+          </commentPr>
+        </mc:Choice>
+        <mc:Fallback/>
+      </mc:AlternateContent>
     </comment>
     <comment ref="B8" authorId="0">
       <text>
@@ -89,6 +131,27 @@
           <t xml:space="preserve">Sun 4.44; giants ~2; white dwarfs ~8.</t>
         </r>
       </text>
+      <mc:AlternateContent>
+        <mc:Choice Requires="v2">
+          <commentPr autoFill="true" autoScale="false" colHidden="false" locked="false" rowHidden="false" textHAlign="justify" textVAlign="top">
+            <anchor moveWithCells="false" sizeWithCells="false">
+              <xdr:from>
+                <xdr:col>0</xdr:col>
+                <xdr:colOff>79</xdr:colOff>
+                <xdr:row>0</xdr:row>
+                <xdr:rowOff>5</xdr:rowOff>
+              </xdr:from>
+              <xdr:to>
+                <xdr:col>1</xdr:col>
+                <xdr:colOff>-58</xdr:colOff>
+                <xdr:row>4</xdr:row>
+                <xdr:rowOff>1</xdr:rowOff>
+              </xdr:to>
+            </anchor>
+          </commentPr>
+        </mc:Choice>
+        <mc:Fallback/>
+      </mc:AlternateContent>
     </comment>
     <comment ref="B9" authorId="0">
       <text>
@@ -101,13 +164,34 @@
           <t xml:space="preserve">Solar photosphere ~0.03 m^2/kg.</t>
         </r>
       </text>
+      <mc:AlternateContent>
+        <mc:Choice Requires="v2">
+          <commentPr autoFill="true" autoScale="false" colHidden="false" locked="false" rowHidden="false" textHAlign="justify" textVAlign="top">
+            <anchor moveWithCells="false" sizeWithCells="false">
+              <xdr:from>
+                <xdr:col>0</xdr:col>
+                <xdr:colOff>79</xdr:colOff>
+                <xdr:row>0</xdr:row>
+                <xdr:rowOff>5</xdr:rowOff>
+              </xdr:from>
+              <xdr:to>
+                <xdr:col>1</xdr:col>
+                <xdr:colOff>-58</xdr:colOff>
+                <xdr:row>4</xdr:row>
+                <xdr:rowOff>1</xdr:rowOff>
+              </xdr:to>
+            </anchor>
+          </commentPr>
+        </mc:Choice>
+        <mc:Fallback/>
+      </mc:AlternateContent>
     </comment>
   </commentList>
 </comments>
 </file>
 
 <file path=xl/comments11.xml><?xml version="1.0" encoding="utf-8"?>
-<comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
+<comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:v2="http://schemas.openxmlformats.org/spreadsheetml/2006/main/v2" mc:Ignorable="v2">
   <authors>
     <author>Unknown Author</author>
   </authors>
@@ -123,6 +207,27 @@
           <t xml:space="preserve">B = B0 (1 + beta tau). beta = 0: isothermal, no line.</t>
         </r>
       </text>
+      <mc:AlternateContent>
+        <mc:Choice Requires="v2">
+          <commentPr autoFill="true" autoScale="false" colHidden="false" locked="false" rowHidden="false" textHAlign="justify" textVAlign="top">
+            <anchor moveWithCells="false" sizeWithCells="false">
+              <xdr:from>
+                <xdr:col>0</xdr:col>
+                <xdr:colOff>79</xdr:colOff>
+                <xdr:row>0</xdr:row>
+                <xdr:rowOff>5</xdr:rowOff>
+              </xdr:from>
+              <xdr:to>
+                <xdr:col>1</xdr:col>
+                <xdr:colOff>-58</xdr:colOff>
+                <xdr:row>4</xdr:row>
+                <xdr:rowOff>1</xdr:rowOff>
+              </xdr:to>
+            </anchor>
+          </commentPr>
+        </mc:Choice>
+        <mc:Fallback/>
+      </mc:AlternateContent>
     </comment>
     <comment ref="B7" authorId="0">
       <text>
@@ -135,6 +240,27 @@
           <t xml:space="preserve">Try 0.1 (weak), 10 (saturated), 1e5 (damping wings).</t>
         </r>
       </text>
+      <mc:AlternateContent>
+        <mc:Choice Requires="v2">
+          <commentPr autoFill="true" autoScale="false" colHidden="false" locked="false" rowHidden="false" textHAlign="justify" textVAlign="top">
+            <anchor moveWithCells="false" sizeWithCells="false">
+              <xdr:from>
+                <xdr:col>0</xdr:col>
+                <xdr:colOff>79</xdr:colOff>
+                <xdr:row>0</xdr:row>
+                <xdr:rowOff>5</xdr:rowOff>
+              </xdr:from>
+              <xdr:to>
+                <xdr:col>1</xdr:col>
+                <xdr:colOff>-58</xdr:colOff>
+                <xdr:row>4</xdr:row>
+                <xdr:rowOff>1</xdr:rowOff>
+              </xdr:to>
+            </anchor>
+          </commentPr>
+        </mc:Choice>
+        <mc:Fallback/>
+      </mc:AlternateContent>
     </comment>
     <comment ref="B8" authorId="0">
       <text>
@@ -147,6 +273,27 @@
           <t xml:space="preserve">Voigt damping. Set 0 for a pure Gaussian.</t>
         </r>
       </text>
+      <mc:AlternateContent>
+        <mc:Choice Requires="v2">
+          <commentPr autoFill="true" autoScale="false" colHidden="false" locked="false" rowHidden="false" textHAlign="justify" textVAlign="top">
+            <anchor moveWithCells="false" sizeWithCells="false">
+              <xdr:from>
+                <xdr:col>0</xdr:col>
+                <xdr:colOff>79</xdr:colOff>
+                <xdr:row>0</xdr:row>
+                <xdr:rowOff>5</xdr:rowOff>
+              </xdr:from>
+              <xdr:to>
+                <xdr:col>1</xdr:col>
+                <xdr:colOff>-58</xdr:colOff>
+                <xdr:row>4</xdr:row>
+                <xdr:rowOff>1</xdr:rowOff>
+              </xdr:to>
+            </anchor>
+          </commentPr>
+        </mc:Choice>
+        <mc:Fallback/>
+      </mc:AlternateContent>
     </comment>
     <comment ref="B10" authorId="0">
       <text>
@@ -159,13 +306,34 @@
           <t xml:space="preserve">Fe 55.8, Ca 40.1, Na 23.0, H 1.008</t>
         </r>
       </text>
+      <mc:AlternateContent>
+        <mc:Choice Requires="v2">
+          <commentPr autoFill="true" autoScale="false" colHidden="false" locked="false" rowHidden="false" textHAlign="justify" textVAlign="top">
+            <anchor moveWithCells="false" sizeWithCells="false">
+              <xdr:from>
+                <xdr:col>0</xdr:col>
+                <xdr:colOff>79</xdr:colOff>
+                <xdr:row>0</xdr:row>
+                <xdr:rowOff>5</xdr:rowOff>
+              </xdr:from>
+              <xdr:to>
+                <xdr:col>1</xdr:col>
+                <xdr:colOff>-58</xdr:colOff>
+                <xdr:row>4</xdr:row>
+                <xdr:rowOff>1</xdr:rowOff>
+              </xdr:to>
+            </anchor>
+          </commentPr>
+        </mc:Choice>
+        <mc:Fallback/>
+      </mc:AlternateContent>
     </comment>
   </commentList>
 </comments>
 </file>
 
 <file path=xl/comments2.xml><?xml version="1.0" encoding="utf-8"?>
-<comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
+<comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:v2="http://schemas.openxmlformats.org/spreadsheetml/2006/main/v2" mc:Ignorable="v2">
   <authors>
     <author>Unknown Author</author>
   </authors>
@@ -181,6 +349,27 @@
           <t xml:space="preserve">Fraction of the beam removed per km. Try 0.01 to 10.</t>
         </r>
       </text>
+      <mc:AlternateContent>
+        <mc:Choice Requires="v2">
+          <commentPr autoFill="true" autoScale="false" colHidden="false" locked="false" rowHidden="false" textHAlign="justify" textVAlign="top">
+            <anchor moveWithCells="false" sizeWithCells="false">
+              <xdr:from>
+                <xdr:col>0</xdr:col>
+                <xdr:colOff>79</xdr:colOff>
+                <xdr:row>0</xdr:row>
+                <xdr:rowOff>5</xdr:rowOff>
+              </xdr:from>
+              <xdr:to>
+                <xdr:col>1</xdr:col>
+                <xdr:colOff>-58</xdr:colOff>
+                <xdr:row>4</xdr:row>
+                <xdr:rowOff>1</xdr:rowOff>
+              </xdr:to>
+            </anchor>
+          </commentPr>
+        </mc:Choice>
+        <mc:Fallback/>
+      </mc:AlternateContent>
     </comment>
     <comment ref="B7" authorId="0">
       <text>
@@ -193,13 +382,34 @@
           <t xml:space="preserve">Total path through the gas. Try 0.1 to 20.</t>
         </r>
       </text>
+      <mc:AlternateContent>
+        <mc:Choice Requires="v2">
+          <commentPr autoFill="true" autoScale="false" colHidden="false" locked="false" rowHidden="false" textHAlign="justify" textVAlign="top">
+            <anchor moveWithCells="false" sizeWithCells="false">
+              <xdr:from>
+                <xdr:col>0</xdr:col>
+                <xdr:colOff>79</xdr:colOff>
+                <xdr:row>0</xdr:row>
+                <xdr:rowOff>5</xdr:rowOff>
+              </xdr:from>
+              <xdr:to>
+                <xdr:col>1</xdr:col>
+                <xdr:colOff>-58</xdr:colOff>
+                <xdr:row>4</xdr:row>
+                <xdr:rowOff>1</xdr:rowOff>
+              </xdr:to>
+            </anchor>
+          </commentPr>
+        </mc:Choice>
+        <mc:Fallback/>
+      </mc:AlternateContent>
     </comment>
   </commentList>
 </comments>
 </file>
 
 <file path=xl/comments3.xml><?xml version="1.0" encoding="utf-8"?>
-<comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
+<comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:v2="http://schemas.openxmlformats.org/spreadsheetml/2006/main/v2" mc:Ignorable="v2">
   <authors>
     <author>Unknown Author</author>
   </authors>
@@ -215,6 +425,27 @@
           <t xml:space="preserve">Sun 5772 K; Sirius A 9940 K.</t>
         </r>
       </text>
+      <mc:AlternateContent>
+        <mc:Choice Requires="v2">
+          <commentPr autoFill="true" autoScale="false" colHidden="false" locked="false" rowHidden="false" textHAlign="justify" textVAlign="top">
+            <anchor moveWithCells="false" sizeWithCells="false">
+              <xdr:from>
+                <xdr:col>0</xdr:col>
+                <xdr:colOff>79</xdr:colOff>
+                <xdr:row>0</xdr:row>
+                <xdr:rowOff>5</xdr:rowOff>
+              </xdr:from>
+              <xdr:to>
+                <xdr:col>1</xdr:col>
+                <xdr:colOff>-58</xdr:colOff>
+                <xdr:row>4</xdr:row>
+                <xdr:rowOff>1</xdr:rowOff>
+              </xdr:to>
+            </anchor>
+          </commentPr>
+        </mc:Choice>
+        <mc:Fallback/>
+      </mc:AlternateContent>
     </comment>
     <comment ref="B7" authorId="0">
       <text>
@@ -227,6 +458,27 @@
           <t xml:space="preserve">Sun 1; Sirius A 1.711.</t>
         </r>
       </text>
+      <mc:AlternateContent>
+        <mc:Choice Requires="v2">
+          <commentPr autoFill="true" autoScale="false" colHidden="false" locked="false" rowHidden="false" textHAlign="justify" textVAlign="top">
+            <anchor moveWithCells="false" sizeWithCells="false">
+              <xdr:from>
+                <xdr:col>0</xdr:col>
+                <xdr:colOff>79</xdr:colOff>
+                <xdr:row>0</xdr:row>
+                <xdr:rowOff>5</xdr:rowOff>
+              </xdr:from>
+              <xdr:to>
+                <xdr:col>1</xdr:col>
+                <xdr:colOff>-58</xdr:colOff>
+                <xdr:row>4</xdr:row>
+                <xdr:rowOff>1</xdr:rowOff>
+              </xdr:to>
+            </anchor>
+          </commentPr>
+        </mc:Choice>
+        <mc:Fallback/>
+      </mc:AlternateContent>
     </comment>
     <comment ref="B8" authorId="0">
       <text>
@@ -239,13 +491,34 @@
           <t xml:space="preserve">Earth 1 AU, Mars 1.524 AU, Sirius 543900 AU.</t>
         </r>
       </text>
+      <mc:AlternateContent>
+        <mc:Choice Requires="v2">
+          <commentPr autoFill="true" autoScale="false" colHidden="false" locked="false" rowHidden="false" textHAlign="justify" textVAlign="top">
+            <anchor moveWithCells="false" sizeWithCells="false">
+              <xdr:from>
+                <xdr:col>0</xdr:col>
+                <xdr:colOff>79</xdr:colOff>
+                <xdr:row>0</xdr:row>
+                <xdr:rowOff>5</xdr:rowOff>
+              </xdr:from>
+              <xdr:to>
+                <xdr:col>1</xdr:col>
+                <xdr:colOff>-58</xdr:colOff>
+                <xdr:row>4</xdr:row>
+                <xdr:rowOff>1</xdr:rowOff>
+              </xdr:to>
+            </anchor>
+          </commentPr>
+        </mc:Choice>
+        <mc:Fallback/>
+      </mc:AlternateContent>
     </comment>
   </commentList>
 </comments>
 </file>
 
 <file path=xl/comments4.xml><?xml version="1.0" encoding="utf-8"?>
-<comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
+<comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:v2="http://schemas.openxmlformats.org/spreadsheetml/2006/main/v2" mc:Ignorable="v2">
   <authors>
     <author>Unknown Author</author>
   </authors>
@@ -261,6 +534,27 @@
           <t xml:space="preserve">Try 3000 (red dwarf), 5772 (Sun), 10000 (A star), 30000 (O star).</t>
         </r>
       </text>
+      <mc:AlternateContent>
+        <mc:Choice Requires="v2">
+          <commentPr autoFill="true" autoScale="false" colHidden="false" locked="false" rowHidden="false" textHAlign="justify" textVAlign="top">
+            <anchor moveWithCells="false" sizeWithCells="false">
+              <xdr:from>
+                <xdr:col>0</xdr:col>
+                <xdr:colOff>79</xdr:colOff>
+                <xdr:row>0</xdr:row>
+                <xdr:rowOff>5</xdr:rowOff>
+              </xdr:from>
+              <xdr:to>
+                <xdr:col>1</xdr:col>
+                <xdr:colOff>-58</xdr:colOff>
+                <xdr:row>4</xdr:row>
+                <xdr:rowOff>1</xdr:rowOff>
+              </xdr:to>
+            </anchor>
+          </commentPr>
+        </mc:Choice>
+        <mc:Fallback/>
+      </mc:AlternateContent>
     </comment>
     <comment ref="B7" authorId="0">
       <text>
@@ -273,13 +567,34 @@
           <t xml:space="preserve">Second curve on the chart.</t>
         </r>
       </text>
+      <mc:AlternateContent>
+        <mc:Choice Requires="v2">
+          <commentPr autoFill="true" autoScale="false" colHidden="false" locked="false" rowHidden="false" textHAlign="justify" textVAlign="top">
+            <anchor moveWithCells="false" sizeWithCells="false">
+              <xdr:from>
+                <xdr:col>0</xdr:col>
+                <xdr:colOff>79</xdr:colOff>
+                <xdr:row>0</xdr:row>
+                <xdr:rowOff>5</xdr:rowOff>
+              </xdr:from>
+              <xdr:to>
+                <xdr:col>1</xdr:col>
+                <xdr:colOff>-58</xdr:colOff>
+                <xdr:row>4</xdr:row>
+                <xdr:rowOff>1</xdr:rowOff>
+              </xdr:to>
+            </anchor>
+          </commentPr>
+        </mc:Choice>
+        <mc:Fallback/>
+      </mc:AlternateContent>
     </comment>
   </commentList>
 </comments>
 </file>
 
 <file path=xl/comments5.xml><?xml version="1.0" encoding="utf-8"?>
-<comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
+<comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:v2="http://schemas.openxmlformats.org/spreadsheetml/2006/main/v2" mc:Ignorable="v2">
   <authors>
     <author>Unknown Author</author>
   </authors>
@@ -295,6 +610,27 @@
           <t xml:space="preserve">Mass of the sphere in solar masses.</t>
         </r>
       </text>
+      <mc:AlternateContent>
+        <mc:Choice Requires="v2">
+          <commentPr autoFill="true" autoScale="false" colHidden="false" locked="false" rowHidden="false" textHAlign="justify" textVAlign="top">
+            <anchor moveWithCells="false" sizeWithCells="false">
+              <xdr:from>
+                <xdr:col>0</xdr:col>
+                <xdr:colOff>79</xdr:colOff>
+                <xdr:row>0</xdr:row>
+                <xdr:rowOff>5</xdr:rowOff>
+              </xdr:from>
+              <xdr:to>
+                <xdr:col>1</xdr:col>
+                <xdr:colOff>-58</xdr:colOff>
+                <xdr:row>4</xdr:row>
+                <xdr:rowOff>1</xdr:rowOff>
+              </xdr:to>
+            </anchor>
+          </commentPr>
+        </mc:Choice>
+        <mc:Fallback/>
+      </mc:AlternateContent>
     </comment>
     <comment ref="B8" authorId="0">
       <text>
@@ -307,6 +643,27 @@
           <t xml:space="preserve">Sets the electrons per unit mass: mu_e = 2/(1+X).</t>
         </r>
       </text>
+      <mc:AlternateContent>
+        <mc:Choice Requires="v2">
+          <commentPr autoFill="true" autoScale="false" colHidden="false" locked="false" rowHidden="false" textHAlign="justify" textVAlign="top">
+            <anchor moveWithCells="false" sizeWithCells="false">
+              <xdr:from>
+                <xdr:col>0</xdr:col>
+                <xdr:colOff>79</xdr:colOff>
+                <xdr:row>0</xdr:row>
+                <xdr:rowOff>5</xdr:rowOff>
+              </xdr:from>
+              <xdr:to>
+                <xdr:col>1</xdr:col>
+                <xdr:colOff>-58</xdr:colOff>
+                <xdr:row>4</xdr:row>
+                <xdr:rowOff>1</xdr:rowOff>
+              </xdr:to>
+            </anchor>
+          </commentPr>
+        </mc:Choice>
+        <mc:Fallback/>
+      </mc:AlternateContent>
     </comment>
     <comment ref="B9" authorId="0">
       <text>
@@ -319,13 +676,34 @@
           <t xml:space="preserve">Probability that an interaction destroys the photon (absorption).</t>
         </r>
       </text>
+      <mc:AlternateContent>
+        <mc:Choice Requires="v2">
+          <commentPr autoFill="true" autoScale="false" colHidden="false" locked="false" rowHidden="false" textHAlign="justify" textVAlign="top">
+            <anchor moveWithCells="false" sizeWithCells="false">
+              <xdr:from>
+                <xdr:col>0</xdr:col>
+                <xdr:colOff>79</xdr:colOff>
+                <xdr:row>0</xdr:row>
+                <xdr:rowOff>5</xdr:rowOff>
+              </xdr:from>
+              <xdr:to>
+                <xdr:col>1</xdr:col>
+                <xdr:colOff>-58</xdr:colOff>
+                <xdr:row>4</xdr:row>
+                <xdr:rowOff>1</xdr:rowOff>
+              </xdr:to>
+            </anchor>
+          </commentPr>
+        </mc:Choice>
+        <mc:Fallback/>
+      </mc:AlternateContent>
     </comment>
   </commentList>
 </comments>
 </file>
 
 <file path=xl/comments6.xml><?xml version="1.0" encoding="utf-8"?>
-<comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
+<comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:v2="http://schemas.openxmlformats.org/spreadsheetml/2006/main/v2" mc:Ignorable="v2">
   <authors>
     <author>Unknown Author</author>
   </authors>
@@ -341,6 +719,27 @@
           <t xml:space="preserve">Brightness of the beam entering the slab, in units of S.</t>
         </r>
       </text>
+      <mc:AlternateContent>
+        <mc:Choice Requires="v2">
+          <commentPr autoFill="true" autoScale="false" colHidden="false" locked="false" rowHidden="false" textHAlign="justify" textVAlign="top">
+            <anchor moveWithCells="false" sizeWithCells="false">
+              <xdr:from>
+                <xdr:col>0</xdr:col>
+                <xdr:colOff>79</xdr:colOff>
+                <xdr:row>0</xdr:row>
+                <xdr:rowOff>17</xdr:rowOff>
+              </xdr:from>
+              <xdr:to>
+                <xdr:col>1</xdr:col>
+                <xdr:colOff>-58</xdr:colOff>
+                <xdr:row>4</xdr:row>
+                <xdr:rowOff>13</xdr:rowOff>
+              </xdr:to>
+            </anchor>
+          </commentPr>
+        </mc:Choice>
+        <mc:Fallback/>
+      </mc:AlternateContent>
     </comment>
     <comment ref="B11" authorId="0">
       <text>
@@ -353,6 +752,27 @@
           <t xml:space="preserve">Hot, optically thick base.</t>
         </r>
       </text>
+      <mc:AlternateContent>
+        <mc:Choice Requires="v2">
+          <commentPr autoFill="true" autoScale="false" colHidden="false" locked="false" rowHidden="false" textHAlign="justify" textVAlign="top">
+            <anchor moveWithCells="false" sizeWithCells="false">
+              <xdr:from>
+                <xdr:col>0</xdr:col>
+                <xdr:colOff>79</xdr:colOff>
+                <xdr:row>0</xdr:row>
+                <xdr:rowOff>17</xdr:rowOff>
+              </xdr:from>
+              <xdr:to>
+                <xdr:col>1</xdr:col>
+                <xdr:colOff>-58</xdr:colOff>
+                <xdr:row>4</xdr:row>
+                <xdr:rowOff>13</xdr:rowOff>
+              </xdr:to>
+            </anchor>
+          </commentPr>
+        </mc:Choice>
+        <mc:Fallback/>
+      </mc:AlternateContent>
     </comment>
     <comment ref="B12" authorId="0">
       <text>
@@ -365,6 +785,27 @@
           <t xml:space="preserve">Make it larger than T_base for a thermal inversion.</t>
         </r>
       </text>
+      <mc:AlternateContent>
+        <mc:Choice Requires="v2">
+          <commentPr autoFill="true" autoScale="false" colHidden="false" locked="false" rowHidden="false" textHAlign="justify" textVAlign="top">
+            <anchor moveWithCells="false" sizeWithCells="false">
+              <xdr:from>
+                <xdr:col>0</xdr:col>
+                <xdr:colOff>79</xdr:colOff>
+                <xdr:row>0</xdr:row>
+                <xdr:rowOff>17</xdr:rowOff>
+              </xdr:from>
+              <xdr:to>
+                <xdr:col>1</xdr:col>
+                <xdr:colOff>-58</xdr:colOff>
+                <xdr:row>4</xdr:row>
+                <xdr:rowOff>13</xdr:rowOff>
+              </xdr:to>
+            </anchor>
+          </commentPr>
+        </mc:Choice>
+        <mc:Fallback/>
+      </mc:AlternateContent>
     </comment>
     <comment ref="B13" authorId="0">
       <text>
@@ -377,6 +818,27 @@
           <t xml:space="preserve">Optical depth at the centre of H-alpha. Try 0.1 to 100.</t>
         </r>
       </text>
+      <mc:AlternateContent>
+        <mc:Choice Requires="v2">
+          <commentPr autoFill="true" autoScale="false" colHidden="false" locked="false" rowHidden="false" textHAlign="justify" textVAlign="top">
+            <anchor moveWithCells="false" sizeWithCells="false">
+              <xdr:from>
+                <xdr:col>0</xdr:col>
+                <xdr:colOff>79</xdr:colOff>
+                <xdr:row>0</xdr:row>
+                <xdr:rowOff>17</xdr:rowOff>
+              </xdr:from>
+              <xdr:to>
+                <xdr:col>1</xdr:col>
+                <xdr:colOff>-58</xdr:colOff>
+                <xdr:row>4</xdr:row>
+                <xdr:rowOff>13</xdr:rowOff>
+              </xdr:to>
+            </anchor>
+          </commentPr>
+        </mc:Choice>
+        <mc:Fallback/>
+      </mc:AlternateContent>
     </comment>
     <comment ref="B15" authorId="0">
       <text>
@@ -389,13 +851,34 @@
           <t xml:space="preserve">Use 0 for a thin cloud seen against empty sky.</t>
         </r>
       </text>
+      <mc:AlternateContent>
+        <mc:Choice Requires="v2">
+          <commentPr autoFill="true" autoScale="false" colHidden="false" locked="false" rowHidden="false" textHAlign="justify" textVAlign="top">
+            <anchor moveWithCells="false" sizeWithCells="false">
+              <xdr:from>
+                <xdr:col>0</xdr:col>
+                <xdr:colOff>79</xdr:colOff>
+                <xdr:row>0</xdr:row>
+                <xdr:rowOff>17</xdr:rowOff>
+              </xdr:from>
+              <xdr:to>
+                <xdr:col>1</xdr:col>
+                <xdr:colOff>-58</xdr:colOff>
+                <xdr:row>4</xdr:row>
+                <xdr:rowOff>13</xdr:rowOff>
+              </xdr:to>
+            </anchor>
+          </commentPr>
+        </mc:Choice>
+        <mc:Fallback/>
+      </mc:AlternateContent>
     </comment>
   </commentList>
 </comments>
 </file>
 
 <file path=xl/comments7.xml><?xml version="1.0" encoding="utf-8"?>
-<comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
+<comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:v2="http://schemas.openxmlformats.org/spreadsheetml/2006/main/v2" mc:Ignorable="v2">
   <authors>
     <author>Unknown Author</author>
   </authors>
@@ -411,6 +894,27 @@
           <t xml:space="preserve">Try 5772 (Sun), 9900 (A0 star), 20000 (B star).</t>
         </r>
       </text>
+      <mc:AlternateContent>
+        <mc:Choice Requires="v2">
+          <commentPr autoFill="true" autoScale="false" colHidden="false" locked="false" rowHidden="false" textHAlign="justify" textVAlign="top">
+            <anchor moveWithCells="false" sizeWithCells="false">
+              <xdr:from>
+                <xdr:col>0</xdr:col>
+                <xdr:colOff>79</xdr:colOff>
+                <xdr:row>0</xdr:row>
+                <xdr:rowOff>5</xdr:rowOff>
+              </xdr:from>
+              <xdr:to>
+                <xdr:col>1</xdr:col>
+                <xdr:colOff>-58</xdr:colOff>
+                <xdr:row>4</xdr:row>
+                <xdr:rowOff>1</xdr:rowOff>
+              </xdr:to>
+            </anchor>
+          </commentPr>
+        </mc:Choice>
+        <mc:Fallback/>
+      </mc:AlternateContent>
     </comment>
     <comment ref="B7" authorId="0">
       <text>
@@ -423,13 +927,34 @@
           <t xml:space="preserve">Typical photospheres: 1 to 100 Pa.</t>
         </r>
       </text>
+      <mc:AlternateContent>
+        <mc:Choice Requires="v2">
+          <commentPr autoFill="true" autoScale="false" colHidden="false" locked="false" rowHidden="false" textHAlign="justify" textVAlign="top">
+            <anchor moveWithCells="false" sizeWithCells="false">
+              <xdr:from>
+                <xdr:col>0</xdr:col>
+                <xdr:colOff>79</xdr:colOff>
+                <xdr:row>0</xdr:row>
+                <xdr:rowOff>5</xdr:rowOff>
+              </xdr:from>
+              <xdr:to>
+                <xdr:col>1</xdr:col>
+                <xdr:colOff>-58</xdr:colOff>
+                <xdr:row>4</xdr:row>
+                <xdr:rowOff>1</xdr:rowOff>
+              </xdr:to>
+            </anchor>
+          </commentPr>
+        </mc:Choice>
+        <mc:Fallback/>
+      </mc:AlternateContent>
     </comment>
   </commentList>
 </comments>
 </file>
 
 <file path=xl/comments8.xml><?xml version="1.0" encoding="utf-8"?>
-<comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
+<comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:v2="http://schemas.openxmlformats.org/spreadsheetml/2006/main/v2" mc:Ignorable="v2">
   <authors>
     <author>Unknown Author</author>
   </authors>
@@ -445,6 +970,27 @@
           <t xml:space="preserve">Solar 500 nm: a = 0.36 with b = 0.64.</t>
         </r>
       </text>
+      <mc:AlternateContent>
+        <mc:Choice Requires="v2">
+          <commentPr autoFill="true" autoScale="false" colHidden="false" locked="false" rowHidden="false" textHAlign="justify" textVAlign="top">
+            <anchor moveWithCells="false" sizeWithCells="false">
+              <xdr:from>
+                <xdr:col>0</xdr:col>
+                <xdr:colOff>79</xdr:colOff>
+                <xdr:row>0</xdr:row>
+                <xdr:rowOff>5</xdr:rowOff>
+              </xdr:from>
+              <xdr:to>
+                <xdr:col>1</xdr:col>
+                <xdr:colOff>-58</xdr:colOff>
+                <xdr:row>4</xdr:row>
+                <xdr:rowOff>1</xdr:rowOff>
+              </xdr:to>
+            </anchor>
+          </commentPr>
+        </mc:Choice>
+        <mc:Fallback/>
+      </mc:AlternateContent>
     </comment>
     <comment ref="B7" authorId="0">
       <text>
@@ -457,6 +1003,27 @@
           <t xml:space="preserve">b &gt; 0: S increases inward -&gt; limb darkening. b &lt; 0: limb brightening.</t>
         </r>
       </text>
+      <mc:AlternateContent>
+        <mc:Choice Requires="v2">
+          <commentPr autoFill="true" autoScale="false" colHidden="false" locked="false" rowHidden="false" textHAlign="justify" textVAlign="top">
+            <anchor moveWithCells="false" sizeWithCells="false">
+              <xdr:from>
+                <xdr:col>0</xdr:col>
+                <xdr:colOff>79</xdr:colOff>
+                <xdr:row>0</xdr:row>
+                <xdr:rowOff>5</xdr:rowOff>
+              </xdr:from>
+              <xdr:to>
+                <xdr:col>1</xdr:col>
+                <xdr:colOff>-58</xdr:colOff>
+                <xdr:row>4</xdr:row>
+                <xdr:rowOff>1</xdr:rowOff>
+              </xdr:to>
+            </anchor>
+          </commentPr>
+        </mc:Choice>
+        <mc:Fallback/>
+      </mc:AlternateContent>
     </comment>
     <comment ref="B8" authorId="0">
       <text>
@@ -469,13 +1036,34 @@
           <t xml:space="preserve">c = 0 makes Eddington-Barbier exact.</t>
         </r>
       </text>
+      <mc:AlternateContent>
+        <mc:Choice Requires="v2">
+          <commentPr autoFill="true" autoScale="false" colHidden="false" locked="false" rowHidden="false" textHAlign="justify" textVAlign="top">
+            <anchor moveWithCells="false" sizeWithCells="false">
+              <xdr:from>
+                <xdr:col>0</xdr:col>
+                <xdr:colOff>79</xdr:colOff>
+                <xdr:row>0</xdr:row>
+                <xdr:rowOff>5</xdr:rowOff>
+              </xdr:from>
+              <xdr:to>
+                <xdr:col>1</xdr:col>
+                <xdr:colOff>-58</xdr:colOff>
+                <xdr:row>4</xdr:row>
+                <xdr:rowOff>1</xdr:rowOff>
+              </xdr:to>
+            </anchor>
+          </commentPr>
+        </mc:Choice>
+        <mc:Fallback/>
+      </mc:AlternateContent>
     </comment>
   </commentList>
 </comments>
 </file>
 
 <file path=xl/comments9.xml><?xml version="1.0" encoding="utf-8"?>
-<comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
+<comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:v2="http://schemas.openxmlformats.org/spreadsheetml/2006/main/v2" mc:Ignorable="v2">
   <authors>
     <author>Unknown Author</author>
   </authors>
@@ -491,6 +1079,27 @@
           <t xml:space="preserve">1 = pure absorption (LTE). Try 0.1, 0.01, 0.001.</t>
         </r>
       </text>
+      <mc:AlternateContent>
+        <mc:Choice Requires="v2">
+          <commentPr autoFill="true" autoScale="false" colHidden="false" locked="false" rowHidden="false" textHAlign="justify" textVAlign="top">
+            <anchor moveWithCells="false" sizeWithCells="false">
+              <xdr:from>
+                <xdr:col>0</xdr:col>
+                <xdr:colOff>79</xdr:colOff>
+                <xdr:row>0</xdr:row>
+                <xdr:rowOff>5</xdr:rowOff>
+              </xdr:from>
+              <xdr:to>
+                <xdr:col>1</xdr:col>
+                <xdr:colOff>-58</xdr:colOff>
+                <xdr:row>4</xdr:row>
+                <xdr:rowOff>1</xdr:rowOff>
+              </xdr:to>
+            </anchor>
+          </commentPr>
+        </mc:Choice>
+        <mc:Fallback/>
+      </mc:AlternateContent>
     </comment>
   </commentList>
 </comments>
@@ -502,7 +1111,7 @@
     <t xml:space="preserve">Radiative Transfer Lab (spreadsheet edition)</t>
   </si>
   <si>
-    <t xml:space="preserve">Companion to the course 'Radiative Transfer: a graduated course for pre-master students'. One sheet per lecture.</t>
+    <t xml:space="preserve">Companion to the two courses 'Radiative Transfer' (RT1-RT6) and 'Stellar Atmospheres' (SA1-SA5). One sheet per experiment, labelled with its lecture.</t>
   </si>
   <si>
     <t xml:space="preserve">How to use</t>
@@ -547,25 +1156,25 @@
     <t xml:space="preserve">Beam attenuation, optical depth, magnitudes of extinction</t>
   </si>
   <si>
-    <t xml:space="preserve">RT2 Intensity</t>
+    <t xml:space="preserve">RT1 Intensity</t>
   </si>
   <si>
     <t xml:space="preserve">Flux falls as 1/d^2, solid angle too: intensity is conserved</t>
   </si>
   <si>
-    <t xml:space="preserve">RT3 Planck</t>
+    <t xml:space="preserve">RT2 Planck</t>
   </si>
   <si>
     <t xml:space="preserve">Black-body spectrum, Wien peak, Stefan-Boltzmann, RJ and Wien limits</t>
   </si>
   <si>
-    <t xml:space="preserve">RT4 Random walk</t>
+    <t xml:space="preserve">RT2 Random walk</t>
   </si>
   <si>
     <t xml:space="preserve">Mean free path, photon diffusion time, thermalisation depth</t>
   </si>
   <si>
-    <t xml:space="preserve">RT5 Slab &amp; MIT star</t>
+    <t xml:space="preserve">RT3 Slab &amp; MIT star</t>
   </si>
   <si>
     <t xml:space="preserve">Slab solution; MIT two-layer star with Balmer + Paschen lines; thermal inversion</t>
@@ -577,25 +1186,25 @@
     <t xml:space="preserve">Hydrogen ionisation and n=2 population; why Balmer lines peak in A stars</t>
   </si>
   <si>
-    <t xml:space="preserve">RT7 Eddington-Barbier</t>
+    <t xml:space="preserve">RT4 Eddington-Barbier</t>
   </si>
   <si>
     <t xml:space="preserve">Emergent intensity, limb darkening, Eddington-Barbier error</t>
   </si>
   <si>
-    <t xml:space="preserve">RT8 Scattering</t>
+    <t xml:space="preserve">RT4 Scattering</t>
   </si>
   <si>
     <t xml:space="preserve">S = eps B + (1-eps) J: Eddington solution, sqrt(eps) law; Rosseland mean calculator</t>
   </si>
   <si>
-    <t xml:space="preserve">SA5 Gray atmosphere</t>
+    <t xml:space="preserve">SA4 Gray atmosphere</t>
   </si>
   <si>
     <t xml:space="preserve">Exact gray LTE model: T(tau), limb darkening at any wavelength, emergent spectrum, pressure</t>
   </si>
   <si>
-    <t xml:space="preserve">SA6 Lines</t>
+    <t xml:space="preserve">SA4 Lines</t>
   </si>
   <si>
     <t xml:space="preserve">Milne-Eddington LTE line profile and curve of growth</t>
@@ -667,7 +1276,7 @@
     <t xml:space="preserve">I(s)/I(0)</t>
   </si>
   <si>
-    <t xml:space="preserve">Lecture RT2 - Why a star looks equally bright per square arcsecond from any distance</t>
+    <t xml:space="preserve">Lecture RT1 - Why a star looks equally bright per square arcsecond from any distance</t>
   </si>
   <si>
     <t xml:space="preserve">Flux falls as 1/d^2, but the solid angle of the star falls in exactly the same way: their ratio, the intensity, is constant.</t>
@@ -745,7 +1354,7 @@
     <t xml:space="preserve">I / I_surface</t>
   </si>
   <si>
-    <t xml:space="preserve">Lecture RT3 - How a black body changes with temperature</t>
+    <t xml:space="preserve">Lecture RT2 - How a black body changes with temperature</t>
   </si>
   <si>
     <t xml:space="preserve">Raise T: the peak moves to shorter wavelengths (Wien) and the total flux grows as T^4 (Stefan-Boltzmann).</t>
@@ -799,7 +1408,7 @@
     <t xml:space="preserve">Wien</t>
   </si>
   <si>
-    <t xml:space="preserve">Lecture RT4 - How long does light take to leave a star?</t>
+    <t xml:space="preserve">Lecture RT2 - How long does light take to leave a star?</t>
   </si>
   <si>
     <t xml:space="preserve">A scattered photon random-walks: after N steps of length l it is only sqrt(N) l away, so escaping from optical depth tau takes N ~ tau^2 steps.</t>
@@ -877,7 +1486,7 @@
     <t xml:space="preserve">escape chance ~ exp(-tau sqrt(3 eps))</t>
   </si>
   <si>
-    <t xml:space="preserve">Lecture RT5 - Absorption or emission lines? A slab and the MIT 8.901 two-layer star</t>
+    <t xml:space="preserve">Lecture RT3 - Absorption or emission lines? A slab and the MIT 8.901 two-layer star</t>
   </si>
   <si>
     <t xml:space="preserve">The beam relaxes toward the source function. Lines are dark if the gas in front is cooler than the background, bright if hotter.</t>
@@ -1018,7 +1627,7 @@
     <t xml:space="preserve">N2/N_total x 1e5</t>
   </si>
   <si>
-    <t xml:space="preserve">Lecture RT7 - What depth do we see at each point of the stellar disk?</t>
+    <t xml:space="preserve">Lecture RT4 - What depth do we see at each point of the stellar disk?</t>
   </si>
   <si>
     <t xml:space="preserve">The emergent intensity is S averaged with weight exp(-tau/mu)/mu. Eddington-Barbier: I(0,mu) ~ S(tau = mu), exact for linear S.</t>
@@ -1069,7 +1678,7 @@
     <t xml:space="preserve">weight exp(-tau/mu)/mu</t>
   </si>
   <si>
-    <t xml:space="preserve">Lecture RT8 - Why is S below B at the surface of an isothermal scattering atmosphere?</t>
+    <t xml:space="preserve">Lecture RT4 - Why is S below B at the surface of an isothermal scattering atmosphere?</t>
   </si>
   <si>
     <t xml:space="preserve">Photons scatter ~1/eps times before destruction and leak out within tau ~ 1/sqrt(eps) of the surface, so J and S fall below B there.</t>
@@ -1132,7 +1741,7 @@
     <t xml:space="preserve">Planck-type mean (arithmetic)</t>
   </si>
   <si>
-    <t xml:space="preserve">Lecture SA5 - The complete gray LTE atmosphere</t>
+    <t xml:space="preserve">Lecture SA4 - The complete gray LTE atmosphere</t>
   </si>
   <si>
     <t xml:space="preserve">Exact solution (Hopf q, Chandrasekhar H) vs Eddington. The model scales with T_eff; limb darkening and spectrum are integrated numerically.</t>
@@ -1213,7 +1822,7 @@
     <t xml:space="preserve">pi B_lambda(T_eff)</t>
   </si>
   <si>
-    <t xml:space="preserve">Lecture SA6 - How does a spectral line grow? Milne-Eddington profiles and the curve of growth</t>
+    <t xml:space="preserve">Lecture SA4 - How does a spectral line grow? Milne-Eddington profiles and the curve of growth</t>
   </si>
   <si>
     <t xml:space="preserve">In LTE a line is dark because we see higher, cooler layers at its frequencies. Saturation: the core cannot drop below 1/(1+2beta/3).</t>
@@ -2223,11 +2832,11 @@
           </c:yVal>
           <c:smooth val="0"/>
         </c:ser>
-        <c:axId val="55305833"/>
-        <c:axId val="55375249"/>
+        <c:axId val="32607907"/>
+        <c:axId val="4105414"/>
       </c:scatterChart>
       <c:valAx>
-        <c:axId val="55305833"/>
+        <c:axId val="32607907"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -2303,12 +2912,12 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="55375249"/>
+        <c:crossAx val="4105414"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="midCat"/>
       </c:valAx>
       <c:valAx>
-        <c:axId val="55375249"/>
+        <c:axId val="4105414"/>
         <c:scaling>
           <c:orientation val="minMax"/>
           <c:max val="1"/>
@@ -2386,7 +2995,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="55305833"/>
+        <c:crossAx val="32607907"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="midCat"/>
       </c:valAx>
@@ -4181,11 +4790,11 @@
           </c:yVal>
           <c:smooth val="0"/>
         </c:ser>
-        <c:axId val="82484130"/>
-        <c:axId val="29187508"/>
+        <c:axId val="94098732"/>
+        <c:axId val="25155581"/>
       </c:scatterChart>
       <c:valAx>
-        <c:axId val="82484130"/>
+        <c:axId val="94098732"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -4261,12 +4870,12 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="29187508"/>
+        <c:crossAx val="25155581"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="midCat"/>
       </c:valAx>
       <c:valAx>
-        <c:axId val="29187508"/>
+        <c:axId val="25155581"/>
         <c:scaling>
           <c:orientation val="minMax"/>
           <c:min val="0"/>
@@ -4343,7 +4952,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="82484130"/>
+        <c:crossAx val="94098732"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="midCat"/>
       </c:valAx>
@@ -4494,7 +5103,7 @@
           </c:dLbls>
           <c:xVal>
             <c:numRef>
-              <c:f>'RT7 Eddington-Barbier'!$E$20:$E$40</c:f>
+              <c:f>'RT4 Eddington-Barbier'!$E$20:$E$40</c:f>
               <c:numCache>
                 <c:formatCode>0.00</c:formatCode>
                 <c:ptCount val="21"/>
@@ -4566,7 +5175,7 @@
           </c:xVal>
           <c:yVal>
             <c:numRef>
-              <c:f>'RT7 Eddington-Barbier'!$F$20:$F$40</c:f>
+              <c:f>'RT4 Eddington-Barbier'!$F$20:$F$40</c:f>
               <c:numCache>
                 <c:formatCode>0.0000</c:formatCode>
                 <c:ptCount val="21"/>
@@ -4638,11 +5247,11 @@
           </c:yVal>
           <c:smooth val="0"/>
         </c:ser>
-        <c:axId val="49703797"/>
-        <c:axId val="16589848"/>
+        <c:axId val="26976167"/>
+        <c:axId val="7416438"/>
       </c:scatterChart>
       <c:valAx>
-        <c:axId val="49703797"/>
+        <c:axId val="26976167"/>
         <c:scaling>
           <c:orientation val="minMax"/>
           <c:max val="1"/>
@@ -4720,12 +5329,12 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="16589848"/>
+        <c:crossAx val="7416438"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="midCat"/>
       </c:valAx>
       <c:valAx>
-        <c:axId val="16589848"/>
+        <c:axId val="7416438"/>
         <c:scaling>
           <c:orientation val="minMax"/>
           <c:min val="0"/>
@@ -4802,7 +5411,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="49703797"/>
+        <c:crossAx val="26976167"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="midCat"/>
       </c:valAx>
@@ -4953,7 +5562,7 @@
           </c:dLbls>
           <c:xVal>
             <c:numRef>
-              <c:f>'RT7 Eddington-Barbier'!$H$20:$H$60</c:f>
+              <c:f>'RT4 Eddington-Barbier'!$H$20:$H$60</c:f>
               <c:numCache>
                 <c:formatCode>0.000</c:formatCode>
                 <c:ptCount val="41"/>
@@ -5085,7 +5694,7 @@
           </c:xVal>
           <c:yVal>
             <c:numRef>
-              <c:f>'RT7 Eddington-Barbier'!$I$20:$I$60</c:f>
+              <c:f>'RT4 Eddington-Barbier'!$I$20:$I$60</c:f>
               <c:numCache>
                 <c:formatCode>0.0000</c:formatCode>
                 <c:ptCount val="41"/>
@@ -5217,11 +5826,11 @@
           </c:yVal>
           <c:smooth val="0"/>
         </c:ser>
-        <c:axId val="62386877"/>
-        <c:axId val="21674412"/>
+        <c:axId val="10219871"/>
+        <c:axId val="1885089"/>
       </c:scatterChart>
       <c:valAx>
-        <c:axId val="62386877"/>
+        <c:axId val="10219871"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -5297,12 +5906,12 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="21674412"/>
+        <c:crossAx val="1885089"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="midCat"/>
       </c:valAx>
       <c:valAx>
-        <c:axId val="21674412"/>
+        <c:axId val="1885089"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -5378,7 +5987,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="62386877"/>
+        <c:crossAx val="10219871"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="midCat"/>
       </c:valAx>
@@ -5529,7 +6138,7 @@
           </c:dLbls>
           <c:xVal>
             <c:numRef>
-              <c:f>'RT7 Eddington-Barbier'!$H$20:$H$60</c:f>
+              <c:f>'RT4 Eddington-Barbier'!$H$20:$H$60</c:f>
               <c:numCache>
                 <c:formatCode>0.000</c:formatCode>
                 <c:ptCount val="41"/>
@@ -5661,7 +6270,7 @@
           </c:xVal>
           <c:yVal>
             <c:numRef>
-              <c:f>'RT7 Eddington-Barbier'!$J$20:$J$60</c:f>
+              <c:f>'RT4 Eddington-Barbier'!$J$20:$J$60</c:f>
               <c:numCache>
                 <c:formatCode>0.0000</c:formatCode>
                 <c:ptCount val="41"/>
@@ -5793,11 +6402,11 @@
           </c:yVal>
           <c:smooth val="0"/>
         </c:ser>
-        <c:axId val="23419116"/>
-        <c:axId val="80925745"/>
+        <c:axId val="17045295"/>
+        <c:axId val="57552872"/>
       </c:scatterChart>
       <c:valAx>
-        <c:axId val="23419116"/>
+        <c:axId val="17045295"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -5873,12 +6482,12 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="80925745"/>
+        <c:crossAx val="57552872"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="midCat"/>
       </c:valAx>
       <c:valAx>
-        <c:axId val="80925745"/>
+        <c:axId val="57552872"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -5954,7 +6563,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="23419116"/>
+        <c:crossAx val="17045295"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="midCat"/>
       </c:valAx>
@@ -6105,7 +6714,7 @@
           </c:dLbls>
           <c:xVal>
             <c:numRef>
-              <c:f>'RT8 Scattering'!$E$17:$E$69</c:f>
+              <c:f>'RT4 Scattering'!$E$17:$E$69</c:f>
               <c:numCache>
                 <c:formatCode>0.000E+00</c:formatCode>
                 <c:ptCount val="53"/>
@@ -6273,7 +6882,7 @@
           </c:xVal>
           <c:yVal>
             <c:numRef>
-              <c:f>'RT8 Scattering'!$F$17:$F$69</c:f>
+              <c:f>'RT4 Scattering'!$F$17:$F$69</c:f>
               <c:numCache>
                 <c:formatCode>0.0000</c:formatCode>
                 <c:ptCount val="53"/>
@@ -6497,7 +7106,7 @@
           </c:dLbls>
           <c:xVal>
             <c:numRef>
-              <c:f>'RT8 Scattering'!$E$17:$E$69</c:f>
+              <c:f>'RT4 Scattering'!$E$17:$E$69</c:f>
               <c:numCache>
                 <c:formatCode>0.000E+00</c:formatCode>
                 <c:ptCount val="53"/>
@@ -6665,7 +7274,7 @@
           </c:xVal>
           <c:yVal>
             <c:numRef>
-              <c:f>'RT8 Scattering'!$G$17:$G$69</c:f>
+              <c:f>'RT4 Scattering'!$G$17:$G$69</c:f>
               <c:numCache>
                 <c:formatCode>0.0000</c:formatCode>
                 <c:ptCount val="53"/>
@@ -6833,11 +7442,11 @@
           </c:yVal>
           <c:smooth val="0"/>
         </c:ser>
-        <c:axId val="99705898"/>
-        <c:axId val="97062796"/>
+        <c:axId val="57148572"/>
+        <c:axId val="83867156"/>
       </c:scatterChart>
       <c:valAx>
-        <c:axId val="99705898"/>
+        <c:axId val="57148572"/>
         <c:scaling>
           <c:logBase val="10"/>
           <c:orientation val="minMax"/>
@@ -6914,12 +7523,12 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="97062796"/>
+        <c:crossAx val="83867156"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="midCat"/>
       </c:valAx>
       <c:valAx>
-        <c:axId val="97062796"/>
+        <c:axId val="83867156"/>
         <c:scaling>
           <c:orientation val="minMax"/>
           <c:max val="1"/>
@@ -6997,7 +7606,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="99705898"/>
+        <c:crossAx val="57148572"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="midCat"/>
       </c:valAx>
@@ -7148,7 +7757,7 @@
           </c:dLbls>
           <c:xVal>
             <c:numRef>
-              <c:f>'SA5 Gray atmosphere'!$E$32:$E$101</c:f>
+              <c:f>'SA4 Gray atmosphere'!$E$32:$E$101</c:f>
               <c:numCache>
                 <c:formatCode>0.000E+00</c:formatCode>
                 <c:ptCount val="70"/>
@@ -7367,7 +7976,7 @@
           </c:xVal>
           <c:yVal>
             <c:numRef>
-              <c:f>'SA5 Gray atmosphere'!$I$32:$I$101</c:f>
+              <c:f>'SA4 Gray atmosphere'!$I$32:$I$101</c:f>
               <c:numCache>
                 <c:formatCode>0</c:formatCode>
                 <c:ptCount val="70"/>
@@ -7642,7 +8251,7 @@
           </c:dLbls>
           <c:xVal>
             <c:numRef>
-              <c:f>'SA5 Gray atmosphere'!$E$32:$E$101</c:f>
+              <c:f>'SA4 Gray atmosphere'!$E$32:$E$101</c:f>
               <c:numCache>
                 <c:formatCode>0.000E+00</c:formatCode>
                 <c:ptCount val="70"/>
@@ -7861,7 +8470,7 @@
           </c:xVal>
           <c:yVal>
             <c:numRef>
-              <c:f>'SA5 Gray atmosphere'!$J$32:$J$101</c:f>
+              <c:f>'SA4 Gray atmosphere'!$J$32:$J$101</c:f>
               <c:numCache>
                 <c:formatCode>0</c:formatCode>
                 <c:ptCount val="70"/>
@@ -8080,11 +8689,11 @@
           </c:yVal>
           <c:smooth val="0"/>
         </c:ser>
-        <c:axId val="75758088"/>
-        <c:axId val="85847200"/>
+        <c:axId val="87500168"/>
+        <c:axId val="40134461"/>
       </c:scatterChart>
       <c:valAx>
-        <c:axId val="75758088"/>
+        <c:axId val="87500168"/>
         <c:scaling>
           <c:logBase val="10"/>
           <c:orientation val="minMax"/>
@@ -8161,12 +8770,12 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="85847200"/>
+        <c:crossAx val="40134461"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="midCat"/>
       </c:valAx>
       <c:valAx>
-        <c:axId val="85847200"/>
+        <c:axId val="40134461"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -8242,7 +8851,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="75758088"/>
+        <c:crossAx val="87500168"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="midCat"/>
       </c:valAx>
@@ -8393,7 +9002,7 @@
           </c:dLbls>
           <c:xVal>
             <c:numRef>
-              <c:f>'SA5 Gray atmosphere'!$M$20:$M$40</c:f>
+              <c:f>'SA4 Gray atmosphere'!$M$20:$M$40</c:f>
               <c:numCache>
                 <c:formatCode>0.00</c:formatCode>
                 <c:ptCount val="21"/>
@@ -8465,7 +9074,7 @@
           </c:xVal>
           <c:yVal>
             <c:numRef>
-              <c:f>'SA5 Gray atmosphere'!$O$20:$O$40</c:f>
+              <c:f>'SA4 Gray atmosphere'!$O$20:$O$40</c:f>
               <c:numCache>
                 <c:formatCode>0.0000</c:formatCode>
                 <c:ptCount val="21"/>
@@ -8593,7 +9202,7 @@
           </c:dLbls>
           <c:xVal>
             <c:numRef>
-              <c:f>'SA5 Gray atmosphere'!$M$20:$M$40</c:f>
+              <c:f>'SA4 Gray atmosphere'!$M$20:$M$40</c:f>
               <c:numCache>
                 <c:formatCode>0.00</c:formatCode>
                 <c:ptCount val="21"/>
@@ -8665,7 +9274,7 @@
           </c:xVal>
           <c:yVal>
             <c:numRef>
-              <c:f>'SA5 Gray atmosphere'!$P$20:$P$40</c:f>
+              <c:f>'SA4 Gray atmosphere'!$P$20:$P$40</c:f>
               <c:numCache>
                 <c:formatCode>0.0000</c:formatCode>
                 <c:ptCount val="21"/>
@@ -8793,7 +9402,7 @@
           </c:dLbls>
           <c:xVal>
             <c:numRef>
-              <c:f>'SA5 Gray atmosphere'!$M$20:$M$40</c:f>
+              <c:f>'SA4 Gray atmosphere'!$M$20:$M$40</c:f>
               <c:numCache>
                 <c:formatCode>0.00</c:formatCode>
                 <c:ptCount val="21"/>
@@ -8865,7 +9474,7 @@
           </c:xVal>
           <c:yVal>
             <c:numRef>
-              <c:f>'SA5 Gray atmosphere'!$Q$20:$Q$40</c:f>
+              <c:f>'SA4 Gray atmosphere'!$Q$20:$Q$40</c:f>
               <c:numCache>
                 <c:formatCode>0.0000</c:formatCode>
                 <c:ptCount val="21"/>
@@ -8937,11 +9546,11 @@
           </c:yVal>
           <c:smooth val="0"/>
         </c:ser>
-        <c:axId val="46830083"/>
-        <c:axId val="69113022"/>
+        <c:axId val="83647709"/>
+        <c:axId val="14761341"/>
       </c:scatterChart>
       <c:valAx>
-        <c:axId val="46830083"/>
+        <c:axId val="83647709"/>
         <c:scaling>
           <c:orientation val="minMax"/>
           <c:max val="1"/>
@@ -9019,12 +9628,12 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="69113022"/>
+        <c:crossAx val="14761341"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="midCat"/>
       </c:valAx>
       <c:valAx>
-        <c:axId val="69113022"/>
+        <c:axId val="14761341"/>
         <c:scaling>
           <c:orientation val="minMax"/>
           <c:max val="1"/>
@@ -9102,7 +9711,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="46830083"/>
+        <c:crossAx val="83647709"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="midCat"/>
       </c:valAx>
@@ -9253,7 +9862,7 @@
           </c:dLbls>
           <c:xVal>
             <c:numRef>
-              <c:f>'SA5 Gray atmosphere'!$S$34:$S$144</c:f>
+              <c:f>'SA4 Gray atmosphere'!$S$34:$S$144</c:f>
               <c:numCache>
                 <c:formatCode>0.0</c:formatCode>
                 <c:ptCount val="111"/>
@@ -9595,7 +10204,7 @@
           </c:xVal>
           <c:yVal>
             <c:numRef>
-              <c:f>'SA5 Gray atmosphere'!$T$34:$T$144</c:f>
+              <c:f>'SA4 Gray atmosphere'!$T$34:$T$144</c:f>
               <c:numCache>
                 <c:formatCode>0.000E+00</c:formatCode>
                 <c:ptCount val="111"/>
@@ -9993,7 +10602,7 @@
           </c:dLbls>
           <c:xVal>
             <c:numRef>
-              <c:f>'SA5 Gray atmosphere'!$S$34:$S$144</c:f>
+              <c:f>'SA4 Gray atmosphere'!$S$34:$S$144</c:f>
               <c:numCache>
                 <c:formatCode>0.0</c:formatCode>
                 <c:ptCount val="111"/>
@@ -10335,7 +10944,7 @@
           </c:xVal>
           <c:yVal>
             <c:numRef>
-              <c:f>'SA5 Gray atmosphere'!$V$34:$V$144</c:f>
+              <c:f>'SA4 Gray atmosphere'!$V$34:$V$144</c:f>
               <c:numCache>
                 <c:formatCode>0.000E+00</c:formatCode>
                 <c:ptCount val="111"/>
@@ -10677,11 +11286,11 @@
           </c:yVal>
           <c:smooth val="0"/>
         </c:ser>
-        <c:axId val="34538824"/>
-        <c:axId val="47455286"/>
+        <c:axId val="56528756"/>
+        <c:axId val="28913528"/>
       </c:scatterChart>
       <c:valAx>
-        <c:axId val="34538824"/>
+        <c:axId val="56528756"/>
         <c:scaling>
           <c:logBase val="10"/>
           <c:orientation val="minMax"/>
@@ -10758,12 +11367,12 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="47455286"/>
+        <c:crossAx val="28913528"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="midCat"/>
       </c:valAx>
       <c:valAx>
-        <c:axId val="47455286"/>
+        <c:axId val="28913528"/>
         <c:scaling>
           <c:logBase val="10"/>
           <c:orientation val="minMax"/>
@@ -10840,7 +11449,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="34538824"/>
+        <c:crossAx val="56528756"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="midCat"/>
       </c:valAx>
@@ -10991,7 +11600,7 @@
           </c:dLbls>
           <c:xVal>
             <c:numRef>
-              <c:f>'SA6 Lines'!$E$26:$E$106</c:f>
+              <c:f>'SA4 Lines'!$E$26:$E$106</c:f>
               <c:numCache>
                 <c:formatCode>0.0</c:formatCode>
                 <c:ptCount val="81"/>
@@ -11243,7 +11852,7 @@
           </c:xVal>
           <c:yVal>
             <c:numRef>
-              <c:f>'SA6 Lines'!$F$26:$F$106</c:f>
+              <c:f>'SA4 Lines'!$F$26:$F$106</c:f>
               <c:numCache>
                 <c:formatCode>0.0000</c:formatCode>
                 <c:ptCount val="81"/>
@@ -11495,11 +12104,11 @@
           </c:yVal>
           <c:smooth val="0"/>
         </c:ser>
-        <c:axId val="29722737"/>
-        <c:axId val="81171067"/>
+        <c:axId val="46651933"/>
+        <c:axId val="76463050"/>
       </c:scatterChart>
       <c:valAx>
-        <c:axId val="29722737"/>
+        <c:axId val="46651933"/>
         <c:scaling>
           <c:orientation val="minMax"/>
           <c:max val="8"/>
@@ -11577,12 +12186,12 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="81171067"/>
+        <c:crossAx val="76463050"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="midCat"/>
       </c:valAx>
       <c:valAx>
-        <c:axId val="81171067"/>
+        <c:axId val="76463050"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -11658,7 +12267,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="29722737"/>
+        <c:crossAx val="46651933"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="midCat"/>
       </c:valAx>
@@ -11809,7 +12418,7 @@
           </c:dLbls>
           <c:xVal>
             <c:numRef>
-              <c:f>'SA6 Lines'!$H$26:$H$58</c:f>
+              <c:f>'SA4 Lines'!$H$26:$H$58</c:f>
               <c:numCache>
                 <c:formatCode>0.00E+00</c:formatCode>
                 <c:ptCount val="33"/>
@@ -11917,7 +12526,7 @@
           </c:xVal>
           <c:yVal>
             <c:numRef>
-              <c:f>'SA6 Lines'!$I$26:$I$58</c:f>
+              <c:f>'SA4 Lines'!$I$26:$I$58</c:f>
               <c:numCache>
                 <c:formatCode>0.0000</c:formatCode>
                 <c:ptCount val="33"/>
@@ -12081,7 +12690,7 @@
           </c:dLbls>
           <c:xVal>
             <c:numRef>
-              <c:f>'SA6 Lines'!$H$26:$H$58</c:f>
+              <c:f>'SA4 Lines'!$H$26:$H$58</c:f>
               <c:numCache>
                 <c:formatCode>0.00E+00</c:formatCode>
                 <c:ptCount val="33"/>
@@ -12189,7 +12798,7 @@
           </c:xVal>
           <c:yVal>
             <c:numRef>
-              <c:f>'SA6 Lines'!$J$26:$J$58</c:f>
+              <c:f>'SA4 Lines'!$J$26:$J$58</c:f>
               <c:numCache>
                 <c:formatCode>0.0000</c:formatCode>
                 <c:ptCount val="33"/>
@@ -12353,7 +12962,7 @@
           </c:dLbls>
           <c:xVal>
             <c:numRef>
-              <c:f>'SA6 Lines'!$H$26:$H$58</c:f>
+              <c:f>'SA4 Lines'!$H$26:$H$58</c:f>
               <c:numCache>
                 <c:formatCode>0.00E+00</c:formatCode>
                 <c:ptCount val="33"/>
@@ -12461,7 +13070,7 @@
           </c:xVal>
           <c:yVal>
             <c:numRef>
-              <c:f>'SA6 Lines'!$K$26:$K$58</c:f>
+              <c:f>'SA4 Lines'!$K$26:$K$58</c:f>
               <c:numCache>
                 <c:formatCode>0.0000</c:formatCode>
                 <c:ptCount val="33"/>
@@ -12569,11 +13178,11 @@
           </c:yVal>
           <c:smooth val="0"/>
         </c:ser>
-        <c:axId val="89772214"/>
-        <c:axId val="11783439"/>
+        <c:axId val="51640941"/>
+        <c:axId val="37481122"/>
       </c:scatterChart>
       <c:valAx>
-        <c:axId val="89772214"/>
+        <c:axId val="51640941"/>
         <c:scaling>
           <c:logBase val="10"/>
           <c:orientation val="minMax"/>
@@ -12650,12 +13259,12 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="11783439"/>
+        <c:crossAx val="37481122"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="midCat"/>
       </c:valAx>
       <c:valAx>
-        <c:axId val="11783439"/>
+        <c:axId val="37481122"/>
         <c:scaling>
           <c:logBase val="10"/>
           <c:orientation val="minMax"/>
@@ -12734,7 +13343,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="89772214"/>
+        <c:crossAx val="51640941"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="midCat"/>
       </c:valAx>
@@ -12885,7 +13494,7 @@
           </c:dLbls>
           <c:xVal>
             <c:numRef>
-              <c:f>'RT2 Intensity'!$E$21:$E$53</c:f>
+              <c:f>'RT1 Intensity'!$E$21:$E$53</c:f>
               <c:numCache>
                 <c:formatCode>0.00E+00</c:formatCode>
                 <c:ptCount val="33"/>
@@ -12993,7 +13602,7 @@
           </c:xVal>
           <c:yVal>
             <c:numRef>
-              <c:f>'RT2 Intensity'!$F$21:$F$53</c:f>
+              <c:f>'RT1 Intensity'!$F$21:$F$53</c:f>
               <c:numCache>
                 <c:formatCode>0.00E+00</c:formatCode>
                 <c:ptCount val="33"/>
@@ -13157,7 +13766,7 @@
           </c:dLbls>
           <c:xVal>
             <c:numRef>
-              <c:f>'RT2 Intensity'!$E$21:$E$53</c:f>
+              <c:f>'RT1 Intensity'!$E$21:$E$53</c:f>
               <c:numCache>
                 <c:formatCode>0.00E+00</c:formatCode>
                 <c:ptCount val="33"/>
@@ -13265,7 +13874,7 @@
           </c:xVal>
           <c:yVal>
             <c:numRef>
-              <c:f>'RT2 Intensity'!$H$21:$H$53</c:f>
+              <c:f>'RT1 Intensity'!$H$21:$H$53</c:f>
               <c:numCache>
                 <c:formatCode>0</c:formatCode>
                 <c:ptCount val="33"/>
@@ -13373,11 +13982,11 @@
           </c:yVal>
           <c:smooth val="0"/>
         </c:ser>
-        <c:axId val="77784081"/>
-        <c:axId val="10426368"/>
+        <c:axId val="60181612"/>
+        <c:axId val="17782534"/>
       </c:scatterChart>
       <c:valAx>
-        <c:axId val="77784081"/>
+        <c:axId val="60181612"/>
         <c:scaling>
           <c:logBase val="10"/>
           <c:orientation val="minMax"/>
@@ -13454,12 +14063,12 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="10426368"/>
+        <c:crossAx val="17782534"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="midCat"/>
       </c:valAx>
       <c:valAx>
-        <c:axId val="10426368"/>
+        <c:axId val="17782534"/>
         <c:scaling>
           <c:logBase val="10"/>
           <c:orientation val="minMax"/>
@@ -13537,7 +14146,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="77784081"/>
+        <c:crossAx val="60181612"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="midCat"/>
       </c:valAx>
@@ -13688,7 +14297,7 @@
           </c:dLbls>
           <c:xVal>
             <c:numRef>
-              <c:f>'RT3 Planck'!$E$18:$E$77</c:f>
+              <c:f>'RT2 Planck'!$E$18:$E$77</c:f>
               <c:numCache>
                 <c:formatCode>0.0</c:formatCode>
                 <c:ptCount val="60"/>
@@ -13877,7 +14486,7 @@
           </c:xVal>
           <c:yVal>
             <c:numRef>
-              <c:f>'RT3 Planck'!$F$18:$F$77</c:f>
+              <c:f>'RT2 Planck'!$F$18:$F$77</c:f>
               <c:numCache>
                 <c:formatCode>0.000E+00</c:formatCode>
                 <c:ptCount val="60"/>
@@ -14122,7 +14731,7 @@
           </c:dLbls>
           <c:xVal>
             <c:numRef>
-              <c:f>'RT3 Planck'!$E$18:$E$77</c:f>
+              <c:f>'RT2 Planck'!$E$18:$E$77</c:f>
               <c:numCache>
                 <c:formatCode>0.0</c:formatCode>
                 <c:ptCount val="60"/>
@@ -14311,7 +14920,7 @@
           </c:xVal>
           <c:yVal>
             <c:numRef>
-              <c:f>'RT3 Planck'!$G$18:$G$77</c:f>
+              <c:f>'RT2 Planck'!$G$18:$G$77</c:f>
               <c:numCache>
                 <c:formatCode>0.000E+00</c:formatCode>
                 <c:ptCount val="60"/>
@@ -14500,11 +15109,11 @@
           </c:yVal>
           <c:smooth val="0"/>
         </c:ser>
-        <c:axId val="97253950"/>
-        <c:axId val="76239142"/>
+        <c:axId val="8374578"/>
+        <c:axId val="44542293"/>
       </c:scatterChart>
       <c:valAx>
-        <c:axId val="97253950"/>
+        <c:axId val="8374578"/>
         <c:scaling>
           <c:orientation val="minMax"/>
           <c:max val="3000"/>
@@ -14582,12 +15191,12 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="76239142"/>
+        <c:crossAx val="44542293"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="midCat"/>
       </c:valAx>
       <c:valAx>
-        <c:axId val="76239142"/>
+        <c:axId val="44542293"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -14663,7 +15272,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="97253950"/>
+        <c:crossAx val="8374578"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="midCat"/>
       </c:valAx>
@@ -14814,7 +15423,7 @@
           </c:dLbls>
           <c:xVal>
             <c:numRef>
-              <c:f>'RT3 Planck'!$E$18:$E$77</c:f>
+              <c:f>'RT2 Planck'!$E$18:$E$77</c:f>
               <c:numCache>
                 <c:formatCode>0.0</c:formatCode>
                 <c:ptCount val="60"/>
@@ -15003,7 +15612,7 @@
           </c:xVal>
           <c:yVal>
             <c:numRef>
-              <c:f>'RT3 Planck'!$F$18:$F$77</c:f>
+              <c:f>'RT2 Planck'!$F$18:$F$77</c:f>
               <c:numCache>
                 <c:formatCode>0.000E+00</c:formatCode>
                 <c:ptCount val="60"/>
@@ -15248,7 +15857,7 @@
           </c:dLbls>
           <c:xVal>
             <c:numRef>
-              <c:f>'RT3 Planck'!$E$18:$E$77</c:f>
+              <c:f>'RT2 Planck'!$E$18:$E$77</c:f>
               <c:numCache>
                 <c:formatCode>0.0</c:formatCode>
                 <c:ptCount val="60"/>
@@ -15437,7 +16046,7 @@
           </c:xVal>
           <c:yVal>
             <c:numRef>
-              <c:f>'RT3 Planck'!$H$18:$H$77</c:f>
+              <c:f>'RT2 Planck'!$H$18:$H$77</c:f>
               <c:numCache>
                 <c:formatCode>0.000E+00</c:formatCode>
                 <c:ptCount val="60"/>
@@ -15682,7 +16291,7 @@
           </c:dLbls>
           <c:xVal>
             <c:numRef>
-              <c:f>'RT3 Planck'!$E$18:$E$77</c:f>
+              <c:f>'RT2 Planck'!$E$18:$E$77</c:f>
               <c:numCache>
                 <c:formatCode>0.0</c:formatCode>
                 <c:ptCount val="60"/>
@@ -15871,7 +16480,7 @@
           </c:xVal>
           <c:yVal>
             <c:numRef>
-              <c:f>'RT3 Planck'!$I$18:$I$77</c:f>
+              <c:f>'RT2 Planck'!$I$18:$I$77</c:f>
               <c:numCache>
                 <c:formatCode>0.000E+00</c:formatCode>
                 <c:ptCount val="60"/>
@@ -16060,11 +16669,11 @@
           </c:yVal>
           <c:smooth val="0"/>
         </c:ser>
-        <c:axId val="77095345"/>
-        <c:axId val="18615844"/>
+        <c:axId val="87443349"/>
+        <c:axId val="36178552"/>
       </c:scatterChart>
       <c:valAx>
-        <c:axId val="77095345"/>
+        <c:axId val="87443349"/>
         <c:scaling>
           <c:logBase val="10"/>
           <c:orientation val="minMax"/>
@@ -16141,12 +16750,12 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="18615844"/>
+        <c:crossAx val="36178552"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="midCat"/>
       </c:valAx>
       <c:valAx>
-        <c:axId val="18615844"/>
+        <c:axId val="36178552"/>
         <c:scaling>
           <c:logBase val="10"/>
           <c:orientation val="minMax"/>
@@ -16223,7 +16832,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="77095345"/>
+        <c:crossAx val="87443349"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="midCat"/>
       </c:valAx>
@@ -16374,7 +16983,7 @@
           </c:dLbls>
           <c:xVal>
             <c:numRef>
-              <c:f>'RT4 Random walk'!$E$23:$E$52</c:f>
+              <c:f>'RT2 Random walk'!$E$23:$E$52</c:f>
               <c:numCache>
                 <c:formatCode>0</c:formatCode>
                 <c:ptCount val="30"/>
@@ -16473,7 +17082,7 @@
           </c:xVal>
           <c:yVal>
             <c:numRef>
-              <c:f>'RT4 Random walk'!$F$23:$F$52</c:f>
+              <c:f>'RT2 Random walk'!$F$23:$F$52</c:f>
               <c:numCache>
                 <c:formatCode>#,##0</c:formatCode>
                 <c:ptCount val="30"/>
@@ -16572,11 +17181,11 @@
           </c:yVal>
           <c:smooth val="0"/>
         </c:ser>
-        <c:axId val="25006489"/>
-        <c:axId val="50078134"/>
+        <c:axId val="97346656"/>
+        <c:axId val="38452845"/>
       </c:scatterChart>
       <c:valAx>
-        <c:axId val="25006489"/>
+        <c:axId val="97346656"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -16652,12 +17261,12 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="50078134"/>
+        <c:crossAx val="38452845"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="midCat"/>
       </c:valAx>
       <c:valAx>
-        <c:axId val="50078134"/>
+        <c:axId val="38452845"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -16733,7 +17342,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="25006489"/>
+        <c:crossAx val="97346656"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="midCat"/>
       </c:valAx>
@@ -16884,7 +17493,7 @@
           </c:dLbls>
           <c:xVal>
             <c:numRef>
-              <c:f>'RT4 Random walk'!$E$23:$E$52</c:f>
+              <c:f>'RT2 Random walk'!$E$23:$E$52</c:f>
               <c:numCache>
                 <c:formatCode>0</c:formatCode>
                 <c:ptCount val="30"/>
@@ -16983,7 +17592,7 @@
           </c:xVal>
           <c:yVal>
             <c:numRef>
-              <c:f>'RT4 Random walk'!$G$23:$G$52</c:f>
+              <c:f>'RT2 Random walk'!$G$23:$G$52</c:f>
               <c:numCache>
                 <c:formatCode>0.0000</c:formatCode>
                 <c:ptCount val="30"/>
@@ -17082,11 +17691,11 @@
           </c:yVal>
           <c:smooth val="0"/>
         </c:ser>
-        <c:axId val="68042575"/>
-        <c:axId val="94061470"/>
+        <c:axId val="32177355"/>
+        <c:axId val="60273095"/>
       </c:scatterChart>
       <c:valAx>
-        <c:axId val="68042575"/>
+        <c:axId val="32177355"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -17162,12 +17771,12 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="94061470"/>
+        <c:crossAx val="60273095"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="midCat"/>
       </c:valAx>
       <c:valAx>
-        <c:axId val="94061470"/>
+        <c:axId val="60273095"/>
         <c:scaling>
           <c:orientation val="minMax"/>
           <c:max val="1"/>
@@ -17245,7 +17854,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="68042575"/>
+        <c:crossAx val="32177355"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="midCat"/>
       </c:valAx>
@@ -17396,7 +18005,7 @@
           </c:dLbls>
           <c:xVal>
             <c:numRef>
-              <c:f>'RT5 Slab &amp; MIT star'!$E$26:$E$56</c:f>
+              <c:f>'RT3 Slab &amp; MIT star'!$E$26:$E$56</c:f>
               <c:numCache>
                 <c:formatCode>0.00</c:formatCode>
                 <c:ptCount val="31"/>
@@ -17498,7 +18107,7 @@
           </c:xVal>
           <c:yVal>
             <c:numRef>
-              <c:f>'RT5 Slab &amp; MIT star'!$F$26:$F$56</c:f>
+              <c:f>'RT3 Slab &amp; MIT star'!$F$26:$F$56</c:f>
               <c:numCache>
                 <c:formatCode>0.0000</c:formatCode>
                 <c:ptCount val="31"/>
@@ -17656,7 +18265,7 @@
           </c:dLbls>
           <c:xVal>
             <c:numRef>
-              <c:f>'RT5 Slab &amp; MIT star'!$E$26:$E$56</c:f>
+              <c:f>'RT3 Slab &amp; MIT star'!$E$26:$E$56</c:f>
               <c:numCache>
                 <c:formatCode>0.00</c:formatCode>
                 <c:ptCount val="31"/>
@@ -17758,7 +18367,7 @@
           </c:xVal>
           <c:yVal>
             <c:numRef>
-              <c:f>'RT5 Slab &amp; MIT star'!$G$26:$G$56</c:f>
+              <c:f>'RT3 Slab &amp; MIT star'!$G$26:$G$56</c:f>
               <c:numCache>
                 <c:formatCode>0</c:formatCode>
                 <c:ptCount val="31"/>
@@ -17860,11 +18469,11 @@
           </c:yVal>
           <c:smooth val="0"/>
         </c:ser>
-        <c:axId val="40519366"/>
-        <c:axId val="73841220"/>
+        <c:axId val="63769224"/>
+        <c:axId val="75388820"/>
       </c:scatterChart>
       <c:valAx>
-        <c:axId val="40519366"/>
+        <c:axId val="63769224"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -17940,12 +18549,12 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="73841220"/>
+        <c:crossAx val="75388820"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="midCat"/>
       </c:valAx>
       <c:valAx>
-        <c:axId val="73841220"/>
+        <c:axId val="75388820"/>
         <c:scaling>
           <c:orientation val="minMax"/>
           <c:min val="0"/>
@@ -18022,7 +18631,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="40519366"/>
+        <c:crossAx val="63769224"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="midCat"/>
       </c:valAx>
@@ -18173,7 +18782,7 @@
           </c:dLbls>
           <c:xVal>
             <c:numRef>
-              <c:f>'RT5 Slab &amp; MIT star'!$H$26:$H$346</c:f>
+              <c:f>'RT3 Slab &amp; MIT star'!$H$26:$H$346</c:f>
               <c:numCache>
                 <c:formatCode>0</c:formatCode>
                 <c:ptCount val="321"/>
@@ -19145,7 +19754,7 @@
           </c:xVal>
           <c:yVal>
             <c:numRef>
-              <c:f>'RT5 Slab &amp; MIT star'!$J$26:$J$346</c:f>
+              <c:f>'RT3 Slab &amp; MIT star'!$J$26:$J$346</c:f>
               <c:numCache>
                 <c:formatCode>0.00</c:formatCode>
                 <c:ptCount val="321"/>
@@ -20173,7 +20782,7 @@
           </c:dLbls>
           <c:xVal>
             <c:numRef>
-              <c:f>'RT5 Slab &amp; MIT star'!$H$26:$H$346</c:f>
+              <c:f>'RT3 Slab &amp; MIT star'!$H$26:$H$346</c:f>
               <c:numCache>
                 <c:formatCode>0</c:formatCode>
                 <c:ptCount val="321"/>
@@ -21145,7 +21754,7 @@
           </c:xVal>
           <c:yVal>
             <c:numRef>
-              <c:f>'RT5 Slab &amp; MIT star'!$K$26:$K$346</c:f>
+              <c:f>'RT3 Slab &amp; MIT star'!$K$26:$K$346</c:f>
               <c:numCache>
                 <c:formatCode>0.00</c:formatCode>
                 <c:ptCount val="321"/>
@@ -22173,7 +22782,7 @@
           </c:dLbls>
           <c:xVal>
             <c:numRef>
-              <c:f>'RT5 Slab &amp; MIT star'!$H$26:$H$346</c:f>
+              <c:f>'RT3 Slab &amp; MIT star'!$H$26:$H$346</c:f>
               <c:numCache>
                 <c:formatCode>0</c:formatCode>
                 <c:ptCount val="321"/>
@@ -23145,7 +23754,7 @@
           </c:xVal>
           <c:yVal>
             <c:numRef>
-              <c:f>'RT5 Slab &amp; MIT star'!$L$26:$L$346</c:f>
+              <c:f>'RT3 Slab &amp; MIT star'!$L$26:$L$346</c:f>
               <c:numCache>
                 <c:formatCode>0.00</c:formatCode>
                 <c:ptCount val="321"/>
@@ -24117,11 +24726,11 @@
           </c:yVal>
           <c:smooth val="0"/>
         </c:ser>
-        <c:axId val="29653960"/>
-        <c:axId val="60706765"/>
+        <c:axId val="19191217"/>
+        <c:axId val="16478523"/>
       </c:scatterChart>
       <c:valAx>
-        <c:axId val="29653960"/>
+        <c:axId val="19191217"/>
         <c:scaling>
           <c:orientation val="minMax"/>
           <c:max val="1000"/>
@@ -24199,12 +24808,12 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="60706765"/>
+        <c:crossAx val="16478523"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="midCat"/>
       </c:valAx>
       <c:valAx>
-        <c:axId val="60706765"/>
+        <c:axId val="16478523"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -24280,7 +24889,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="29653960"/>
+        <c:crossAx val="19191217"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="midCat"/>
       </c:valAx>
@@ -26075,11 +26684,11 @@
           </c:yVal>
           <c:smooth val="0"/>
         </c:ser>
-        <c:axId val="4680732"/>
-        <c:axId val="98931320"/>
+        <c:axId val="5788534"/>
+        <c:axId val="31707399"/>
       </c:scatterChart>
       <c:valAx>
-        <c:axId val="4680732"/>
+        <c:axId val="5788534"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -26155,12 +26764,12 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="98931320"/>
+        <c:crossAx val="31707399"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="midCat"/>
       </c:valAx>
       <c:valAx>
-        <c:axId val="98931320"/>
+        <c:axId val="31707399"/>
         <c:scaling>
           <c:orientation val="minMax"/>
           <c:max val="1"/>
@@ -26238,7 +26847,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="4680732"/>
+        <c:crossAx val="5788534"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="midCat"/>
       </c:valAx>
@@ -27261,15 +27870,15 @@
   </sheetData>
   <hyperlinks>
     <hyperlink ref="A12" r:id="rId1" location="'RT1%20Optical%20depth'!A1" display="RT1 Optical depth"/>
-    <hyperlink ref="A13" r:id="rId2" location="'RT2%20Intensity'!A1" display="RT2 Intensity"/>
-    <hyperlink ref="A14" r:id="rId3" location="'RT3%20Planck'!A1" display="RT3 Planck"/>
-    <hyperlink ref="A15" r:id="rId4" location="'RT4%20Random%20walk'!A1" display="RT4 Random walk"/>
-    <hyperlink ref="A16" r:id="rId5" location="'RT5%20Slab%20&amp;%20MIT%20star'!A1" display="RT5 Slab &amp; MIT star"/>
+    <hyperlink ref="A13" r:id="rId2" location="'RT1%20Intensity'!A1" display="RT1 Intensity"/>
+    <hyperlink ref="A14" r:id="rId3" location="'RT2%20Planck'!A1" display="RT2 Planck"/>
+    <hyperlink ref="A15" r:id="rId4" location="'RT2%20Random%20walk'!A1" display="RT2 Random walk"/>
+    <hyperlink ref="A16" r:id="rId5" location="'RT3%20Slab%20&amp;%20MIT%20star'!A1" display="RT3 Slab &amp; MIT star"/>
     <hyperlink ref="A17" r:id="rId6" location="'SA1%20Saha-Boltzmann'!A1" display="SA1 Saha-Boltzmann"/>
-    <hyperlink ref="A18" r:id="rId7" location="'RT7%20Eddington-Barbier'!A1" display="RT7 Eddington-Barbier"/>
-    <hyperlink ref="A19" r:id="rId8" location="'RT8%20Scattering'!A1" display="RT8 Scattering"/>
-    <hyperlink ref="A20" r:id="rId9" location="'SA5%20Gray%20atmosphere'!A1" display="SA5 Gray atmosphere"/>
-    <hyperlink ref="A21" r:id="rId10" location="'SA6%20Lines'!A1" display="SA6 Lines"/>
+    <hyperlink ref="A18" r:id="rId7" location="'RT4%20Eddington-Barbier'!A1" display="RT4 Eddington-Barbier"/>
+    <hyperlink ref="A19" r:id="rId8" location="'RT4%20Scattering'!A1" display="RT4 Scattering"/>
+    <hyperlink ref="A20" r:id="rId9" location="'SA4%20Gray%20atmosphere'!A1" display="SA4 Gray atmosphere"/>
+    <hyperlink ref="A21" r:id="rId10" location="'SA4%20Lines'!A1" display="SA4 Lines"/>
     <hyperlink ref="A22" r:id="rId11" location="'Constants'!A1" display="Constants"/>
     <hyperlink ref="A23" r:id="rId12" location="'Data'!A1" display="Data"/>
   </hyperlinks>

</xml_diff>